<commit_message>
test: add Access Control and MockAPI Live Integration modules and regenerate report
</commit_message>
<xml_diff>
--- a/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
+++ b/Employee_management/Emp_Mng/tests/Employee_Management_Test_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="84">
   <si>
     <t>Project name:</t>
   </si>
@@ -40,13 +40,13 @@
     <t>Project Assigned Date:</t>
   </si>
   <si>
-    <t>2026-07-09</t>
+    <t>2026-07-10</t>
   </si>
   <si>
     <t>Module Name:</t>
   </si>
   <si>
-    <t>Employee Directory &amp; Pay Analytics (User Interaction)</t>
+    <t>Employee Directory, Pay Analytics, Access Control &amp; Live API Integration</t>
   </si>
   <si>
     <t>End Date:</t>
@@ -160,6 +160,121 @@
   </si>
   <si>
     <t>As Expected: Computed aggregate spending metrics matched.</t>
+  </si>
+  <si>
+    <t>TC#5</t>
+  </si>
+  <si>
+    <t>Verify default access rights assignment on seeding based on employee roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Seed permissions with various roles: Lead, Developer, and standard role.
+2. Verify Lead gets adminAccess, Developer gets writeAccess, and others get readAccess only.</t>
+  </si>
+  <si>
+    <t>Roles: Lead (ID: 101), Developer (ID: 102), Team Member (ID: 103)</t>
+  </si>
+  <si>
+    <t>Lead: adminAccess &amp; writeAccess &amp; readAccess; Developer: writeAccess &amp; readAccess; Team Member: readAccess only.</t>
+  </si>
+  <si>
+    <t>As Expected: Role-based default permissions seeded correctly.</t>
+  </si>
+  <si>
+    <t>TC#6</t>
+  </si>
+  <si>
+    <t>Verify database write and admin access toggle behavior in local storage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Simulate toggling database write permission for a specific employee.
+2. Verify updated permission status updates and persists in simulated state.</t>
+  </si>
+  <si>
+    <t>Toggle field 'writeAccess' from false to true</t>
+  </si>
+  <si>
+    <t>Permission value is inverted and persisted in updated permissions mapping.</t>
+  </si>
+  <si>
+    <t>As Expected: Toggle correctly inverted permission value and persisted update.</t>
+  </si>
+  <si>
+    <t>TC#7</t>
+  </si>
+  <si>
+    <t>Retrieve standard employee details from live database (Stable Target)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Send HTTP GET request to MockAPI for standard record ID 1.
+2. Validate response code is 200 and fields 'name', 'email', 'department' are present.</t>
+  </si>
+  <si>
+    <t>Endpoint: GET https://6a4b3678f5eab0bb6b6256cf.mockapi.io/Employee/1</t>
+  </si>
+  <si>
+    <t>Response HTTP 200 returned with valid non-empty fields.</t>
+  </si>
+  <si>
+    <t>As Expected: Successfully fetched standard record ID 1. Name: Priya</t>
+  </si>
+  <si>
+    <t>TC#8</t>
+  </si>
+  <si>
+    <t>Validate live API record update operation (Stable Target)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Target standard record ID 2.
+2. Send HTTP PUT request updating salary to 50000.
+3. Verify response status is 200 and returns updated salary.</t>
+  </si>
+  <si>
+    <t>Endpoint: PUT https://6a4b3678f5eab0bb6b6256cf.mockapi.io/Employee/2, data: { salary: 50000 }</t>
+  </si>
+  <si>
+    <t>Response HTTP 200 returned with updated salary set to 50000.</t>
+  </si>
+  <si>
+    <t>As Expected: PUT request succeeded and updated record salary field to 50000.</t>
+  </si>
+  <si>
+    <t>TC#9</t>
+  </si>
+  <si>
+    <t>Validate API response for out-of-bounds record query</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Send GET request for a non-existent or high ID (e.g., 9999).
+2. Verify API returns 404 Not Found error status.</t>
+  </si>
+  <si>
+    <t>Endpoint: GET https://6a4b3678f5eab0bb6b6256cf.mockapi.io/Employee/9999</t>
+  </si>
+  <si>
+    <t>Fetch fails, throwing HTTP error with status 404.</t>
+  </si>
+  <si>
+    <t>As Expected: API correctly returned HTTP 404 for out-of-bounds record ID.</t>
+  </si>
+  <si>
+    <t>TC#10</t>
+  </si>
+  <si>
+    <t>Validate required input fields validation logic during profile creation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Run validateField validation rules on invalid name, invalid email, and negative salary.
+2. Check if validation errors are accurately identified and returned.</t>
+  </si>
+  <si>
+    <t>Fields: Name = 'A' (too short), Email = 'bad_email', Salary = -100</t>
+  </si>
+  <si>
+    <t>Validation functions catch all errors and return correct warning messages.</t>
+  </si>
+  <si>
+    <t>As Expected: Validation logic correctly flagged all invalid inputs.</t>
   </si>
 </sst>
 </file>
@@ -602,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -792,6 +907,144 @@
         <v>28</v>
       </c>
     </row>
+    <row r="15" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>